<commit_message>
Fix vendor for SR 72 (MMK)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4c5Y1XBRj63SkdBZ73bUS
</commit_message>
<xml_diff>
--- a/quotes/Rajby-PO-Compare/Power_and_other_Tools_Rates_less2pct.xlsx
+++ b/quotes/Rajby-PO-Compare/Power_and_other_Tools_Rates_less2pct.xlsx
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="258">
   <si>
     <t xml:space="preserve">Power &amp; other Tools Inquiry - Rates (2% less, rounded to 10)</t>
   </si>
@@ -3429,7 +3429,9 @@
       <c r="F76" s="7" t="n">
         <v>17860</v>
       </c>
-      <c r="G76" s="6"/>
+      <c r="G76" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="H76" s="8" t="n">
         <f aca="false">IF(F76="","",ROUND(F76*(1-$B$2),-1))</f>
         <v>17500</v>

</xml_diff>